<commit_message>
Implement full daily refresh pipeline and publish 2026-03-07 snapshot/report
</commit_message>
<xml_diff>
--- a/model.xlsx
+++ b/model.xlsx
@@ -13912,7 +13912,7 @@
       </c>
       <c r="C24" s="34" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="D24" s="34" t="inlineStr">
@@ -14533,7 +14533,7 @@
         </is>
       </c>
       <c r="B49" s="33" t="n">
-        <v>68228</v>
+        <v>67959</v>
       </c>
       <c r="C49" s="34" t="inlineStr">
         <is>
@@ -14558,7 +14558,7 @@
         </is>
       </c>
       <c r="B50" s="33" t="n">
-        <v>77.38979999999999</v>
+        <v>77.3824</v>
       </c>
       <c r="C50" s="34" t="inlineStr">
         <is>

</xml_diff>